<commit_message>
Add questions: Test Survey
</commit_message>
<xml_diff>
--- a/surveys/test-survey/questions.xlsx
+++ b/surveys/test-survey/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhaight\Python\InterviewGuides\surveys\test-survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D55227A-BDF2-480F-B484-64DEE8783656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7006636E-A67E-4C84-AFD5-7714A270C73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
   <si>
     <t>Survey Settings</t>
   </si>
@@ -59,15 +59,9 @@
     <t>How does your experience relate to this position?</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Walk me through a complex project you completed.</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Competency</t>
   </si>
   <si>
@@ -84,6 +78,12 @@
   </si>
   <si>
     <t>http://www.youtube.com</t>
+  </si>
+  <si>
+    <t>Shared Values</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
@@ -531,15 +531,15 @@
         <v>6</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -583,41 +583,29 @@
       <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -627,41 +615,37 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>14</v>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>